<commit_message>
Auto sync Onetech 31/10/2026 08:44
</commit_message>
<xml_diff>
--- a/data/Thang10/DanhSachChiTietDonHang (2).xlsx
+++ b/data/Thang10/DanhSachChiTietDonHang (2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="159">
   <si>
     <t>BÁO CÁO LINE ITEM</t>
   </si>
@@ -151,36 +151,294 @@
     <t>Công Ty TNHH Minh Phát Thành</t>
   </si>
   <si>
+    <t>26SF.HC22209</t>
+  </si>
+  <si>
+    <t>Mai Thị Linh</t>
+  </si>
+  <si>
+    <t>MIX_LE</t>
+  </si>
+  <si>
+    <t>SM-FM-10KF1326.08</t>
+  </si>
+  <si>
+    <t>W-279314920433717</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>DM-10KF1326.01</t>
+  </si>
+  <si>
+    <t>Nguyễn Út Đèo</t>
+  </si>
+  <si>
+    <t>Đơn hàng giao sau</t>
+  </si>
+  <si>
+    <t>Đã gửi đơn</t>
+  </si>
+  <si>
+    <t>31/10/2026 08:40:43</t>
+  </si>
+  <si>
+    <t>2793149</t>
+  </si>
+  <si>
+    <t>Chị Hiền</t>
+  </si>
+  <si>
+    <t>Ki Ốt 5 Đường 265</t>
+  </si>
+  <si>
+    <t>Hồ Chí Minh</t>
+  </si>
+  <si>
+    <t>P. Tăng Nhơn Phú</t>
+  </si>
+  <si>
+    <t>Refreshment Drinks</t>
+  </si>
+  <si>
+    <t>Nước tăng lực Wake up 247</t>
+  </si>
+  <si>
+    <t>08TL001</t>
+  </si>
+  <si>
+    <t>Nước tăng lực vị cà phê Wake up 247 - 4bl x 6chai x 330ml</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Seasoning</t>
+  </si>
+  <si>
+    <t>Nước mắm Nam Ngư</t>
+  </si>
+  <si>
+    <t>03NM00882</t>
+  </si>
+  <si>
+    <t>Nước mắm Nam Ngư (QR) MN 3bl x 6chai x 750ml</t>
+  </si>
+  <si>
+    <t>Nước mắm Nam Ngư Đệ II</t>
+  </si>
+  <si>
+    <t>03NM00790</t>
+  </si>
+  <si>
+    <t>Nước chấm Nam Ngư Đệ Nhị (QR) 15chai x 900ml</t>
+  </si>
+  <si>
+    <t>Nước mắm Nam Ngư siêu tiết kiệm Can</t>
+  </si>
+  <si>
+    <t>03NM00938</t>
+  </si>
+  <si>
+    <t>Nước chấm Nam Ngư Siêu tiết kiệm (QR) 4chai x 4.8L</t>
+  </si>
+  <si>
+    <t>Nước tương Tam Thái Tử Nhị Ca</t>
+  </si>
+  <si>
+    <t>03NT00537</t>
+  </si>
+  <si>
+    <t>Nước chấm Tam Thái Tử Nhị ca 25chai x 500ml</t>
+  </si>
+  <si>
     <t>26SF.HC22774</t>
   </si>
   <si>
     <t>Ngô Nguyễn Cao Kỳ</t>
   </si>
   <si>
-    <t>MIX_LE</t>
-  </si>
-  <si>
     <t>SM-FM-10KF1326.11</t>
   </si>
   <si>
+    <t>W-285018020433544</t>
+  </si>
+  <si>
+    <t>31/10/2026 08:38:57</t>
+  </si>
+  <si>
+    <t>2850180</t>
+  </si>
+  <si>
+    <t>Tạp Hóa 70D</t>
+  </si>
+  <si>
+    <t>70 D Đường 185</t>
+  </si>
+  <si>
+    <t>P. Phước Long</t>
+  </si>
+  <si>
+    <t>Convenience Foods</t>
+  </si>
+  <si>
+    <t>Mì Kokomi 65</t>
+  </si>
+  <si>
+    <t>02KK00313</t>
+  </si>
+  <si>
+    <t>Mì Kokomi Tôm chua cay 30gói x 65gr</t>
+  </si>
+  <si>
+    <t>Mì trộn Omachi Tô</t>
+  </si>
+  <si>
+    <t>02OM00446</t>
+  </si>
+  <si>
+    <t>Mì Omachi trộn xốt Tôm phô mai trứng muối 12tô x 105gr</t>
+  </si>
+  <si>
+    <t>02OM00447</t>
+  </si>
+  <si>
+    <t>Mì Omachi trộn xốt Spaghetti 12tô x 105gr</t>
+  </si>
+  <si>
+    <t>14SF.HC0198</t>
+  </si>
+  <si>
+    <t>Lê Thị Thơm</t>
+  </si>
+  <si>
+    <t>SM-FM-10KF1326.10</t>
+  </si>
+  <si>
+    <t>W-313725820433418</t>
+  </si>
+  <si>
+    <t>31/10/2026 08:37:28</t>
+  </si>
+  <si>
+    <t>3137258</t>
+  </si>
+  <si>
+    <t>Xe Nước 670</t>
+  </si>
+  <si>
+    <t>670 Đỗ Xuân Hợp</t>
+  </si>
+  <si>
+    <t>Processed Meats</t>
+  </si>
+  <si>
+    <t>Xúc xích Ponnie Bin &amp; Bon</t>
+  </si>
+  <si>
+    <t>02XX00229</t>
+  </si>
+  <si>
+    <t>Xúc xích dinh dưỡng Bin &amp; Bon thịt Heo 20gói x 6cây x 35gr</t>
+  </si>
+  <si>
+    <t>Nước khoáng Lemona có ga</t>
+  </si>
+  <si>
+    <t>08VH039</t>
+  </si>
+  <si>
+    <t>Nước khoáng Lemona có gas tự nhiên 4bl x 6chai x 500ml</t>
+  </si>
+  <si>
+    <t>Nước tương Tam Thái Tử Nhất Ca</t>
+  </si>
+  <si>
+    <t>03NT00380</t>
+  </si>
+  <si>
+    <t>Nước tương Tam Thái Tử Nhất ca iode 4bl x 6chai x 500ml</t>
+  </si>
+  <si>
+    <t>18SF.HC4149</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Bích Trâm</t>
+  </si>
+  <si>
+    <t>SM-FM-10KF1326.14</t>
+  </si>
+  <si>
+    <t>W-99920453620431388</t>
+  </si>
+  <si>
+    <t>31/10/2026 08:15:49</t>
+  </si>
+  <si>
+    <t>999204536</t>
+  </si>
+  <si>
+    <t>Tạp Hoá Nhung</t>
+  </si>
+  <si>
+    <t>192 Bưng Ông Thoàn</t>
+  </si>
+  <si>
+    <t>Xúc xích Ponnie</t>
+  </si>
+  <si>
+    <t>02XX00090</t>
+  </si>
+  <si>
+    <t>Xúc xích tiệt trùng Ponnie vị Heo 20gói x 5cây x 35gr</t>
+  </si>
+  <si>
+    <t>Trà Búp Non Tea 365</t>
+  </si>
+  <si>
+    <t>08TR00038</t>
+  </si>
+  <si>
+    <t>Trà Bupnon TEA365 lài vị chanh 4bl x 6chai x 500ml</t>
+  </si>
+  <si>
+    <t>W-400420430884</t>
+  </si>
+  <si>
+    <t>31/10/2026 08:08:48</t>
+  </si>
+  <si>
+    <t>4004</t>
+  </si>
+  <si>
+    <t>Chị Năm</t>
+  </si>
+  <si>
+    <t>37 Chợ Hiệp Phú</t>
+  </si>
+  <si>
+    <t>Hạt nêm Chinsu</t>
+  </si>
+  <si>
+    <t>03HG00134</t>
+  </si>
+  <si>
+    <t>Hạt nêm CHIN-SU ngọt Tôm thơm thịt MN 6gói x 1.8kg</t>
+  </si>
+  <si>
+    <t>Xốt nhà hàng Chinsu</t>
+  </si>
+  <si>
+    <t>03MR00023</t>
+  </si>
+  <si>
+    <t>Xốt nhà hàng CHIN-SU nướng muối ớt 8hộp x 10túi x 80gr</t>
+  </si>
+  <si>
     <t>W-50673620430606</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>DM-10KF1326.01</t>
-  </si>
-  <si>
-    <t>Nguyễn Út Đèo</t>
-  </si>
-  <si>
-    <t>Đơn hàng giao sau</t>
-  </si>
-  <si>
-    <t>Đã gửi đơn</t>
-  </si>
-  <si>
     <t>31/10/2026 08:04:40</t>
   </si>
   <si>
@@ -193,12 +451,6 @@
     <t>185 Dương Đình Hội</t>
   </si>
   <si>
-    <t>Hồ Chí Minh</t>
-  </si>
-  <si>
-    <t>P. Phước Long</t>
-  </si>
-  <si>
     <t>Coffee</t>
   </si>
   <si>
@@ -211,9 +463,6 @@
     <t>Cà phê VCF 3in1 Gold Original (QR) 12bịch x 40gói x 20gr</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>Café Wake Up Sài Gòn</t>
   </si>
   <si>
@@ -223,9 +472,6 @@
     <t>Cà phê Wake up Sài Gòn (QR) 20bịch x 24gói x 19gr</t>
   </si>
   <si>
-    <t>Convenience Foods</t>
-  </si>
-  <si>
     <t>Mì Kokomi Đại 90</t>
   </si>
   <si>
@@ -242,18 +488,6 @@
   </si>
   <si>
     <t>Mì dinh dưỡng khoai tây Omachi hương vị lẩu tôm càng 30gói x 80gr</t>
-  </si>
-  <si>
-    <t>Refreshment Drinks</t>
-  </si>
-  <si>
-    <t>Nước tăng lực Wake up 247</t>
-  </si>
-  <si>
-    <t>08TL001</t>
-  </si>
-  <si>
-    <t>Nước tăng lực vị cà phê Wake up 247 - 4bl x 6chai x 330ml</t>
   </si>
 </sst>
 </file>
@@ -671,7 +905,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AM9"/>
+  <dimension ref="A1:AM30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -892,40 +1126,40 @@
         <v>65</v>
       </c>
       <c r="Z5" s="4">
-        <v>118300</v>
+        <v>8000</v>
       </c>
       <c r="AA5" s="4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="AB5" s="4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AC5" s="4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="4">
-        <v>0.33</v>
+        <v>10</v>
       </c>
       <c r="AE5" s="4">
-        <v>4</v>
+        <v>240</v>
       </c>
       <c r="AF5" s="4">
-        <v>3.596666666666668</v>
+        <v>92.49839999999992</v>
       </c>
       <c r="AG5" s="5">
-        <v>473200</v>
+        <v>1920000</v>
       </c>
       <c r="AH5" s="5">
-        <v>0</v>
+        <v>19200</v>
       </c>
       <c r="AI5" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ5" s="5">
-        <v>473200</v>
+        <v>1900800</v>
       </c>
       <c r="AK5" s="5">
-        <v>473200</v>
+        <v>1900800</v>
       </c>
       <c r="AL5" s="4" t="s">
         <v>66</v>
@@ -999,40 +1233,40 @@
         <v>61</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="X6" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Y6" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Z6" s="4">
-        <v>47300</v>
+        <v>44500</v>
       </c>
       <c r="AA6" s="4">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="AB6" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC6" s="4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AD6" s="4">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AE6" s="4">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="AF6" s="4">
-        <v>5.15</v>
+        <v>17.100000000000005</v>
       </c>
       <c r="AG6" s="5">
-        <v>473000</v>
+        <v>801000</v>
       </c>
       <c r="AH6" s="5">
         <v>0</v>
@@ -1041,10 +1275,10 @@
         <v>0</v>
       </c>
       <c r="AJ6" s="5">
-        <v>473000</v>
+        <v>801000</v>
       </c>
       <c r="AK6" s="5">
-        <v>473000</v>
+        <v>801000</v>
       </c>
       <c r="AL6" s="4" t="s">
         <v>66</v>
@@ -1118,7 +1352,7 @@
         <v>61</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="W7" s="4" t="s">
         <v>71</v>
@@ -1130,28 +1364,28 @@
         <v>73</v>
       </c>
       <c r="Z7" s="4">
-        <v>3833.33334</v>
+        <v>22200</v>
       </c>
       <c r="AA7" s="4">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="AB7" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC7" s="4">
         <v>0</v>
       </c>
       <c r="AD7" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE7" s="4">
-        <v>90</v>
+        <v>15</v>
       </c>
       <c r="AF7" s="4">
-        <v>8.77176</v>
+        <v>16.5</v>
       </c>
       <c r="AG7" s="5">
-        <v>345000.0006</v>
+        <v>333000</v>
       </c>
       <c r="AH7" s="5">
         <v>0</v>
@@ -1160,10 +1394,10 @@
         <v>0</v>
       </c>
       <c r="AJ7" s="5">
-        <v>345000.0006</v>
+        <v>333000</v>
       </c>
       <c r="AK7" s="5">
-        <v>345000.0006</v>
+        <v>333000</v>
       </c>
       <c r="AL7" s="4" t="s">
         <v>66</v>
@@ -1237,7 +1471,7 @@
         <v>61</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="W8" s="4" t="s">
         <v>74</v>
@@ -1249,28 +1483,28 @@
         <v>76</v>
       </c>
       <c r="Z8" s="4">
-        <v>7666.66667</v>
+        <v>62800</v>
       </c>
       <c r="AA8" s="4">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="AB8" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AC8" s="4">
         <v>0</v>
       </c>
       <c r="AD8" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE8" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AF8" s="4">
-        <v>2.7</v>
+        <v>117.99999999999989</v>
       </c>
       <c r="AG8" s="5">
-        <v>230000.0001</v>
+        <v>1256000</v>
       </c>
       <c r="AH8" s="5">
         <v>0</v>
@@ -1279,10 +1513,10 @@
         <v>0</v>
       </c>
       <c r="AJ8" s="5">
-        <v>230000.0001</v>
+        <v>1256000</v>
       </c>
       <c r="AK8" s="5">
-        <v>230000.0001</v>
+        <v>1256000</v>
       </c>
       <c r="AL8" s="4" t="s">
         <v>66</v>
@@ -1356,40 +1590,40 @@
         <v>61</v>
       </c>
       <c r="V9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W9" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="W9" s="4" t="s">
+      <c r="X9" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="X9" s="4" t="s">
+      <c r="Y9" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="Y9" s="4" t="s">
-        <v>80</v>
-      </c>
       <c r="Z9" s="4">
-        <v>8000</v>
+        <v>5952</v>
       </c>
       <c r="AA9" s="4">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AB9" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC9" s="4">
         <v>0</v>
       </c>
       <c r="AD9" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE9" s="4">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="AF9" s="4">
-        <v>18.499679999999984</v>
+        <v>14.575</v>
       </c>
       <c r="AG9" s="5">
-        <v>384000</v>
+        <v>148800</v>
       </c>
       <c r="AH9" s="5">
         <v>0</v>
@@ -1398,15 +1632,2514 @@
         <v>0</v>
       </c>
       <c r="AJ9" s="5">
-        <v>384000</v>
+        <v>148800</v>
       </c>
       <c r="AK9" s="5">
-        <v>384000</v>
+        <v>148800</v>
       </c>
       <c r="AL9" s="4" t="s">
         <v>66</v>
       </c>
       <c r="AM9" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="R10" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="S10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="T10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V10" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="W10" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="X10" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y10" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="Z10" s="4">
+        <v>2583.33334</v>
+      </c>
+      <c r="AA10" s="4">
+        <v>30</v>
+      </c>
+      <c r="AB10" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC10" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE10" s="4">
+        <v>30</v>
+      </c>
+      <c r="AF10" s="4">
+        <v>2.109</v>
+      </c>
+      <c r="AG10" s="5">
+        <v>77500.0002</v>
+      </c>
+      <c r="AH10" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI10" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="5">
+        <v>77500.0002</v>
+      </c>
+      <c r="AK10" s="5">
+        <v>77500.0002</v>
+      </c>
+      <c r="AL10" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM10" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q11" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="R11" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="S11" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="T11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U11" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V11" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="W11" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="X11" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y11" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="Z11" s="4">
+        <v>13000</v>
+      </c>
+      <c r="AA11" s="4">
+        <v>12</v>
+      </c>
+      <c r="AB11" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="4">
+        <v>6</v>
+      </c>
+      <c r="AD11" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="AE11" s="4">
+        <v>6</v>
+      </c>
+      <c r="AF11" s="4">
+        <v>0.979999999999998</v>
+      </c>
+      <c r="AG11" s="5">
+        <v>78000</v>
+      </c>
+      <c r="AH11" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI11" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ11" s="5">
+        <v>78000</v>
+      </c>
+      <c r="AK11" s="5">
+        <v>78000</v>
+      </c>
+      <c r="AL11" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM11" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="S12" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="T12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U12" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V12" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="W12" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="X12" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y12" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z12" s="4">
+        <v>13000</v>
+      </c>
+      <c r="AA12" s="4">
+        <v>12</v>
+      </c>
+      <c r="AB12" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="4">
+        <v>6</v>
+      </c>
+      <c r="AD12" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="AE12" s="4">
+        <v>6</v>
+      </c>
+      <c r="AF12" s="4">
+        <v>0.87</v>
+      </c>
+      <c r="AG12" s="5">
+        <v>78000</v>
+      </c>
+      <c r="AH12" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI12" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ12" s="5">
+        <v>78000</v>
+      </c>
+      <c r="AK12" s="5">
+        <v>78000</v>
+      </c>
+      <c r="AL12" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM12" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="R13" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="S13" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="T13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U13" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V13" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="W13" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="X13" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="Y13" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="Z13" s="4">
+        <v>14000</v>
+      </c>
+      <c r="AA13" s="4">
+        <v>20</v>
+      </c>
+      <c r="AB13" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC13" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE13" s="4">
+        <v>20</v>
+      </c>
+      <c r="AF13" s="4">
+        <v>5.812</v>
+      </c>
+      <c r="AG13" s="5">
+        <v>280000</v>
+      </c>
+      <c r="AH13" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI13" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ13" s="5">
+        <v>280000</v>
+      </c>
+      <c r="AK13" s="5">
+        <v>280000</v>
+      </c>
+      <c r="AL13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM13" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="R14" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="S14" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="T14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U14" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V14" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="W14" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="X14" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="Y14" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z14" s="4">
+        <v>5583.33334</v>
+      </c>
+      <c r="AA14" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB14" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC14" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE14" s="4">
+        <v>24</v>
+      </c>
+      <c r="AF14" s="4">
+        <v>14</v>
+      </c>
+      <c r="AG14" s="5">
+        <v>134000.00016</v>
+      </c>
+      <c r="AH14" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI14" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ14" s="5">
+        <v>134000.00016</v>
+      </c>
+      <c r="AK14" s="5">
+        <v>134000.00016</v>
+      </c>
+      <c r="AL14" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM14" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N15" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="R15" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="S15" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="T15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U15" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V15" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W15" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="X15" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y15" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z15" s="4">
+        <v>22200</v>
+      </c>
+      <c r="AA15" s="4">
+        <v>15</v>
+      </c>
+      <c r="AB15" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC15" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE15" s="4">
+        <v>15</v>
+      </c>
+      <c r="AF15" s="4">
+        <v>16.5</v>
+      </c>
+      <c r="AG15" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AH15" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI15" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ15" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AK15" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AL15" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM15" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="R16" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="S16" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="T16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U16" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V16" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W16" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="X16" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y16" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="Z16" s="4">
+        <v>17500</v>
+      </c>
+      <c r="AA16" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB16" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="4">
+        <v>12</v>
+      </c>
+      <c r="AD16" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="AE16" s="4">
+        <v>12</v>
+      </c>
+      <c r="AF16" s="4">
+        <v>7.149999999999992</v>
+      </c>
+      <c r="AG16" s="5">
+        <v>210000</v>
+      </c>
+      <c r="AH16" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI16" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ16" s="5">
+        <v>210000</v>
+      </c>
+      <c r="AK16" s="5">
+        <v>210000</v>
+      </c>
+      <c r="AL16" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM16" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N17" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q17" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="R17" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="S17" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="T17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U17" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V17" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W17" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="X17" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y17" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z17" s="4">
+        <v>5952</v>
+      </c>
+      <c r="AA17" s="4">
+        <v>25</v>
+      </c>
+      <c r="AB17" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC17" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD17" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE17" s="4">
+        <v>25</v>
+      </c>
+      <c r="AF17" s="4">
+        <v>14.575</v>
+      </c>
+      <c r="AG17" s="5">
+        <v>148800</v>
+      </c>
+      <c r="AH17" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI17" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ17" s="5">
+        <v>148800</v>
+      </c>
+      <c r="AK17" s="5">
+        <v>148800</v>
+      </c>
+      <c r="AL17" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM17" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q18" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="R18" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="S18" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="T18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U18" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V18" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="W18" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="X18" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="Z18" s="4">
+        <v>16400</v>
+      </c>
+      <c r="AA18" s="4">
+        <v>20</v>
+      </c>
+      <c r="AB18" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="4">
+        <v>5</v>
+      </c>
+      <c r="AD18" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="AE18" s="4">
+        <v>5</v>
+      </c>
+      <c r="AF18" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="AG18" s="5">
+        <v>82000</v>
+      </c>
+      <c r="AH18" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI18" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ18" s="5">
+        <v>82000</v>
+      </c>
+      <c r="AK18" s="5">
+        <v>82000</v>
+      </c>
+      <c r="AL18" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM18" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q19" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="R19" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="S19" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="T19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V19" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="W19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="X19" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z19" s="4">
+        <v>8000</v>
+      </c>
+      <c r="AA19" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB19" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC19" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE19" s="4">
+        <v>24</v>
+      </c>
+      <c r="AF19" s="4">
+        <v>9.249839999999992</v>
+      </c>
+      <c r="AG19" s="5">
+        <v>192000</v>
+      </c>
+      <c r="AH19" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ19" s="5">
+        <v>192000</v>
+      </c>
+      <c r="AK19" s="5">
+        <v>192000</v>
+      </c>
+      <c r="AL19" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM19" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q20" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="R20" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="S20" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="T20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U20" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V20" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="W20" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="X20" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y20" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="Z20" s="4">
+        <v>7250</v>
+      </c>
+      <c r="AA20" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB20" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="4">
+        <v>6</v>
+      </c>
+      <c r="AD20" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="AE20" s="4">
+        <v>6</v>
+      </c>
+      <c r="AF20" s="4">
+        <v>3.361499999999996</v>
+      </c>
+      <c r="AG20" s="5">
+        <v>43500</v>
+      </c>
+      <c r="AH20" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI20" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ20" s="5">
+        <v>43500</v>
+      </c>
+      <c r="AK20" s="5">
+        <v>43500</v>
+      </c>
+      <c r="AL20" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM20" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N21" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="O21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q21" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="R21" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="S21" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="T21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U21" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V21" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W21" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="X21" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y21" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z21" s="4">
+        <v>22200</v>
+      </c>
+      <c r="AA21" s="4">
+        <v>15</v>
+      </c>
+      <c r="AB21" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC21" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE21" s="4">
+        <v>15</v>
+      </c>
+      <c r="AF21" s="4">
+        <v>16.5</v>
+      </c>
+      <c r="AG21" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AH21" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI21" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ21" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AK21" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AL21" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM21" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M22" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N22" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q22" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="R22" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="S22" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="T22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U22" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V22" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W22" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="X22" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="Y22" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="Z22" s="4">
+        <v>73600</v>
+      </c>
+      <c r="AA22" s="4">
+        <v>6</v>
+      </c>
+      <c r="AB22" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC22" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE22" s="4">
+        <v>6</v>
+      </c>
+      <c r="AF22" s="4">
+        <v>11.719999999999992</v>
+      </c>
+      <c r="AG22" s="5">
+        <v>441600</v>
+      </c>
+      <c r="AH22" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI22" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ22" s="5">
+        <v>441600</v>
+      </c>
+      <c r="AK22" s="5">
+        <v>441600</v>
+      </c>
+      <c r="AL22" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM22" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N23" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q23" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="R23" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="S23" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="T23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U23" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V23" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W23" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="X23" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y23" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z23" s="4">
+        <v>22200</v>
+      </c>
+      <c r="AA23" s="4">
+        <v>15</v>
+      </c>
+      <c r="AB23" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC23" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE23" s="4">
+        <v>15</v>
+      </c>
+      <c r="AF23" s="4">
+        <v>16.5</v>
+      </c>
+      <c r="AG23" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AH23" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI23" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ23" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AK23" s="5">
+        <v>333000</v>
+      </c>
+      <c r="AL23" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM23" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M24" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N24" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="O24" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P24" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q24" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="R24" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="S24" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="T24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U24" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V24" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W24" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="X24" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y24" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="Z24" s="4">
+        <v>17500</v>
+      </c>
+      <c r="AA24" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB24" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="4">
+        <v>12</v>
+      </c>
+      <c r="AD24" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="AE24" s="4">
+        <v>12</v>
+      </c>
+      <c r="AF24" s="4">
+        <v>7.149999999999992</v>
+      </c>
+      <c r="AG24" s="5">
+        <v>210000</v>
+      </c>
+      <c r="AH24" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI24" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ24" s="5">
+        <v>210000</v>
+      </c>
+      <c r="AK24" s="5">
+        <v>210000</v>
+      </c>
+      <c r="AL24" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM24" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M25" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N25" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P25" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q25" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="R25" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="S25" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="T25" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U25" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V25" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="W25" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="X25" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="Y25" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="Z25" s="4">
+        <v>85000</v>
+      </c>
+      <c r="AA25" s="4">
+        <v>8</v>
+      </c>
+      <c r="AB25" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="4">
+        <v>1</v>
+      </c>
+      <c r="AD25" s="4">
+        <v>0.13</v>
+      </c>
+      <c r="AE25" s="4">
+        <v>1</v>
+      </c>
+      <c r="AF25" s="4">
+        <v>1.3</v>
+      </c>
+      <c r="AG25" s="5">
+        <v>85000</v>
+      </c>
+      <c r="AH25" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI25" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ25" s="5">
+        <v>85000</v>
+      </c>
+      <c r="AK25" s="5">
+        <v>85000</v>
+      </c>
+      <c r="AL25" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM25" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M26" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N26" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P26" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q26" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="R26" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="S26" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="T26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U26" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V26" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="W26" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="X26" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="Y26" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="Z26" s="4">
+        <v>118300</v>
+      </c>
+      <c r="AA26" s="4">
+        <v>12</v>
+      </c>
+      <c r="AB26" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC26" s="4">
+        <v>4</v>
+      </c>
+      <c r="AD26" s="4">
+        <v>0.33</v>
+      </c>
+      <c r="AE26" s="4">
+        <v>4</v>
+      </c>
+      <c r="AF26" s="4">
+        <v>3.596666666666668</v>
+      </c>
+      <c r="AG26" s="5">
+        <v>473200</v>
+      </c>
+      <c r="AH26" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI26" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ26" s="5">
+        <v>473200</v>
+      </c>
+      <c r="AK26" s="5">
+        <v>473200</v>
+      </c>
+      <c r="AL26" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM26" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M27" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N27" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="O27" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P27" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q27" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="R27" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="S27" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="T27" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U27" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V27" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="W27" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="X27" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y27" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="Z27" s="4">
+        <v>47300</v>
+      </c>
+      <c r="AA27" s="4">
+        <v>20</v>
+      </c>
+      <c r="AB27" s="4">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="4">
+        <v>10</v>
+      </c>
+      <c r="AD27" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="AE27" s="4">
+        <v>10</v>
+      </c>
+      <c r="AF27" s="4">
+        <v>5.15</v>
+      </c>
+      <c r="AG27" s="5">
+        <v>473000</v>
+      </c>
+      <c r="AH27" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI27" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ27" s="5">
+        <v>473000</v>
+      </c>
+      <c r="AK27" s="5">
+        <v>473000</v>
+      </c>
+      <c r="AL27" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM27" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M28" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N28" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="O28" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P28" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q28" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="R28" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="S28" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="T28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U28" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V28" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="W28" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="X28" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="Y28" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="Z28" s="4">
+        <v>3833.33334</v>
+      </c>
+      <c r="AA28" s="4">
+        <v>30</v>
+      </c>
+      <c r="AB28" s="4">
+        <v>3</v>
+      </c>
+      <c r="AC28" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="4">
+        <v>3</v>
+      </c>
+      <c r="AE28" s="4">
+        <v>90</v>
+      </c>
+      <c r="AF28" s="4">
+        <v>8.77176</v>
+      </c>
+      <c r="AG28" s="5">
+        <v>345000.0006</v>
+      </c>
+      <c r="AH28" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI28" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ28" s="5">
+        <v>345000.0006</v>
+      </c>
+      <c r="AK28" s="5">
+        <v>345000.0006</v>
+      </c>
+      <c r="AL28" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM28" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L29" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M29" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N29" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="O29" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P29" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q29" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="R29" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="S29" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="T29" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U29" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V29" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="W29" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="X29" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="Y29" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="Z29" s="4">
+        <v>7666.66667</v>
+      </c>
+      <c r="AA29" s="4">
+        <v>30</v>
+      </c>
+      <c r="AB29" s="4">
+        <v>1</v>
+      </c>
+      <c r="AC29" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="4">
+        <v>1</v>
+      </c>
+      <c r="AE29" s="4">
+        <v>30</v>
+      </c>
+      <c r="AF29" s="4">
+        <v>2.7</v>
+      </c>
+      <c r="AG29" s="5">
+        <v>230000.0001</v>
+      </c>
+      <c r="AH29" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ29" s="5">
+        <v>230000.0001</v>
+      </c>
+      <c r="AK29" s="5">
+        <v>230000.0001</v>
+      </c>
+      <c r="AL29" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM29" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L30" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M30" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="N30" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P30" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q30" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="R30" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="S30" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="T30" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U30" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="V30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="W30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="X30" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y30" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z30" s="4">
+        <v>8000</v>
+      </c>
+      <c r="AA30" s="4">
+        <v>24</v>
+      </c>
+      <c r="AB30" s="4">
+        <v>2</v>
+      </c>
+      <c r="AC30" s="4">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="4">
+        <v>2</v>
+      </c>
+      <c r="AE30" s="4">
+        <v>48</v>
+      </c>
+      <c r="AF30" s="4">
+        <v>18.499679999999984</v>
+      </c>
+      <c r="AG30" s="5">
+        <v>384000</v>
+      </c>
+      <c r="AH30" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI30" s="4">
+        <v>0</v>
+      </c>
+      <c r="AJ30" s="5">
+        <v>384000</v>
+      </c>
+      <c r="AK30" s="5">
+        <v>384000</v>
+      </c>
+      <c r="AL30" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM30" s="5">
         <v>0</v>
       </c>
     </row>

</xml_diff>